<commit_message>
feat: rescue card modifiers (#64)
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF6FAD9-600A-4D02-ADB0-7F9607AA552F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F7A40A-3752-4C06-83AB-BAFE40D224DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,9 @@
     <sheet name="Characters" sheetId="3" r:id="rId3"/>
     <sheet name="Thunderbirds" sheetId="4" r:id="rId4"/>
     <sheet name="Pod Vehicles" sheetId="5" r:id="rId5"/>
-    <sheet name="Map Edges" sheetId="7" r:id="rId6"/>
+    <sheet name="Map Edges" sheetId="8" r:id="rId6"/>
+    <sheet name="F.A.B. Cards" sheetId="6" r:id="rId7"/>
+    <sheet name="Event Cards" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="135">
   <si>
     <t>Name</t>
   </si>
@@ -343,6 +345,102 @@
     <t>Rockquake!</t>
   </si>
   <si>
+    <t>The Hood Interferes</t>
+  </si>
+  <si>
+    <t>Explosion on Tracy Island</t>
+  </si>
+  <si>
+    <t>Pod Hydraulics Sabotaged</t>
+  </si>
+  <si>
+    <t>Attack of the Zombites</t>
+  </si>
+  <si>
+    <t>Accidental Injury</t>
+  </si>
+  <si>
+    <t>Rocket Malfunction</t>
+  </si>
+  <si>
+    <t>Kyrano… Kyrano!!</t>
+  </si>
+  <si>
+    <t>Emergency Comms Interrupted</t>
+  </si>
+  <si>
+    <t>USN Sentinel Missile Strike</t>
+  </si>
+  <si>
+    <t>Master of Disguise</t>
+  </si>
+  <si>
+    <t>Icelandic Volcano Eruption</t>
+  </si>
+  <si>
+    <t>Underwater Sealing Unit</t>
+  </si>
+  <si>
+    <t>Holiday in Bonga Bonga</t>
+  </si>
+  <si>
+    <t>Mobile Command Unit</t>
+  </si>
+  <si>
+    <t>Astronaut Spacewalk</t>
+  </si>
+  <si>
+    <t>Grandma's Cooking</t>
+  </si>
+  <si>
+    <t>Experimental Fuel</t>
+  </si>
+  <si>
+    <t>Air Sea Rescue Centre</t>
+  </si>
+  <si>
+    <t>Help from Braman</t>
+  </si>
+  <si>
+    <t>Powder Compact Radio</t>
+  </si>
+  <si>
+    <t>Automatic Camera Detector</t>
+  </si>
+  <si>
+    <t>Tracy Brothers' Portraits</t>
+  </si>
+  <si>
+    <t>Agent-47 Jeremiah Tuttle</t>
+  </si>
+  <si>
+    <t>FAB 1 Hydrofoils</t>
+  </si>
+  <si>
+    <t>Remote Control Hover Camera</t>
+  </si>
+  <si>
+    <t>Personal Hoverjet</t>
+  </si>
+  <si>
+    <t>Sir Jeremy Hodge</t>
+  </si>
+  <si>
+    <t>Long-Range Walkie Talkies</t>
+  </si>
+  <si>
+    <t>Jeff's Orders</t>
+  </si>
+  <si>
+    <t>The Hood's Hypnotic Eyes</t>
+  </si>
+  <si>
+    <t>Edge 1</t>
+  </si>
+  <si>
+    <t>Edge 2</t>
+  </si>
+  <si>
     <t>Domain</t>
   </si>
   <si>
@@ -350,12 +448,6 @@
   </si>
   <si>
     <t>Top Speed</t>
-  </si>
-  <si>
-    <t>Edge 1</t>
-  </si>
-  <si>
-    <t>Edge 2</t>
   </si>
 </sst>
 </file>
@@ -1907,7 +1999,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1915,7 +2007,7 @@
         <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1923,7 +2015,7 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1931,7 +2023,7 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1939,7 +2031,7 @@
         <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1947,7 +2039,7 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1955,7 +2047,7 @@
         <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1963,7 +2055,7 @@
         <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1971,7 +2063,7 @@
         <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1979,7 +2071,7 @@
         <v>67</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1987,7 +2079,7 @@
         <v>88</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -1995,7 +2087,7 @@
         <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2150,10 +2242,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="C1" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2161,7 +2253,7 @@
         <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C2">
         <v>3</v>
@@ -2172,7 +2264,7 @@
         <v>97</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -2194,7 +2286,7 @@
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -2216,7 +2308,7 @@
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -2293,19 +2385,19 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E42479-0211-470A-B268-566711210746}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B37DDD8-053B-497B-A0FD-20F208B606C5}">
   <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="B1" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2316,7 +2408,7 @@
         <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2327,7 +2419,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2338,7 +2430,7 @@
         <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2349,7 +2441,7 @@
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2360,7 +2452,7 @@
         <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2371,7 +2463,7 @@
         <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2382,7 +2474,7 @@
         <v>86</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2393,7 +2485,7 @@
         <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2404,7 +2496,7 @@
         <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2415,7 +2507,7 @@
         <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2426,7 +2518,7 @@
         <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2437,7 +2529,7 @@
         <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2448,7 +2540,7 @@
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -2459,7 +2551,7 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2470,7 +2562,7 @@
         <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2481,7 +2573,7 @@
         <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2492,7 +2584,7 @@
         <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -2503,7 +2595,7 @@
         <v>88</v>
       </c>
       <c r="C19" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -2514,7 +2606,7 @@
         <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2525,7 +2617,7 @@
         <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2536,7 +2628,7 @@
         <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2547,7 +2639,7 @@
         <v>67</v>
       </c>
       <c r="C23" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2625,6 +2717,186 @@
       </c>
       <c r="C30" t="s">
         <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A0DC219-ECA6-4590-958F-6BDC2A6EF2E8}">
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA6DCDF-51E7-4440-B5D3-A355F5D584CF}">
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>